<commit_message>
Add AI test case designer: drafts plan-format cases from a feature spec
</commit_message>
<xml_diff>
--- a/Test_Cases.xlsx
+++ b/Test_Cases.xlsx
@@ -10,7 +10,7 @@
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="4" documentId="11_EB556F077ACD5DCDDE524178BC6F2C9CB50EBC7A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{69D02F28-A40F-4DF6-B1F1-4F3995BECA84}"/>
   <bookViews>
-    <workbookView xWindow="-103" yWindow="-103" windowWidth="16663" windowHeight="9772" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="19440" windowHeight="10320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="1" r:id="rId1"/>
@@ -1045,7 +1045,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -1090,9 +1090,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1472,7 +1469,7 @@
       <c r="I2" s="11" t="s">
         <v>19</v>
       </c>
-      <c r="J2" s="20" t="s">
+      <c r="J2" s="11" t="s">
         <v>269</v>
       </c>
       <c r="K2" s="11"/>

</xml_diff>